<commit_message>
finalized the pcb schematics
</commit_message>
<xml_diff>
--- a/hardware/BOM/External hardware components.xlsx
+++ b/hardware/BOM/External hardware components.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" codeName="ThisWorkbook" defaultThemeVersion="164011"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="8010" windowHeight="7800" tabRatio="477" firstSheet="1" activeTab="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="8010" windowHeight="7800" tabRatio="477"/>
   </bookViews>
   <sheets>
     <sheet name="(Large) EXTERNAL COMPONENTS" sheetId="4" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="140" uniqueCount="123">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="145" uniqueCount="127">
   <si>
     <t>Component</t>
   </si>
@@ -389,6 +389,18 @@
   </si>
   <si>
     <t>Mechanical check valve</t>
+  </si>
+  <si>
+    <t>LEDs</t>
+  </si>
+  <si>
+    <t>OLED Display</t>
+  </si>
+  <si>
+    <t>Graphic LCD Display Module White OLED - Passive Matrix I2C, SPI 0.96" (24.38mm) 128 x 64 [ensure to use I2C]</t>
+  </si>
+  <si>
+    <t>DigiKey [https://www.digikey.com/en/maker/projects/arduino-oled-display-interfacing/0a150e86a90a4743b361376ba0d39722]</t>
   </si>
 </sst>
 </file>
@@ -439,7 +451,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -447,6 +459,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -734,7 +749,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet2"/>
-  <dimension ref="A1:I38"/>
+  <dimension ref="A1:I40"/>
   <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="29.36328125" style="3" customWidth="1"/>
@@ -943,6 +958,9 @@
       <c r="A18" s="1" t="s">
         <v>102</v>
       </c>
+      <c r="B18" s="1">
+        <v>1</v>
+      </c>
       <c r="C18" s="2" t="s">
         <v>69</v>
       </c>
@@ -966,6 +984,9 @@
       <c r="A19" s="1" t="s">
         <v>103</v>
       </c>
+      <c r="B19" s="1">
+        <v>1</v>
+      </c>
       <c r="C19" s="2" t="s">
         <v>74</v>
       </c>
@@ -986,308 +1007,343 @@
       </c>
     </row>
     <row r="20" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A20" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="B20" s="1">
+        <v>2</v>
+      </c>
       <c r="C20" s="2"/>
       <c r="D20" s="2"/>
       <c r="E20" s="2"/>
-      <c r="G20" s="2"/>
-      <c r="H20" s="2"/>
-      <c r="I20" s="2"/>
-    </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A21" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="B21" s="3">
-        <v>1</v>
-      </c>
-      <c r="C21" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="D21" s="3" t="s">
+    </row>
+    <row r="21" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A21" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="B21" s="1">
+        <v>1</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="D21" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="G21" s="3">
-        <v>6.95</v>
-      </c>
-      <c r="H21" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="I21" s="3" t="s">
-        <v>12</v>
-      </c>
+      <c r="E21" s="2">
+        <v>326</v>
+      </c>
+      <c r="G21" s="2">
+        <v>17.5</v>
+      </c>
+      <c r="H21" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="I21" s="5"/>
+    </row>
+    <row r="22" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="C22" s="2"/>
+      <c r="D22" s="2"/>
+      <c r="E22" s="2"/>
+      <c r="G22" s="2"/>
+      <c r="H22" s="2"/>
+      <c r="I22" s="2"/>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A23" s="3" t="s">
-        <v>21</v>
+        <v>5</v>
       </c>
       <c r="B23" s="3">
         <v>1</v>
       </c>
       <c r="C23" s="3" t="s">
-        <v>22</v>
+        <v>3</v>
       </c>
       <c r="D23" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="E23" s="3" t="s">
-        <v>23</v>
+        <v>10</v>
       </c>
       <c r="G23" s="3">
-        <v>34</v>
+        <v>6.95</v>
       </c>
       <c r="H23" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="I23" s="3">
-        <v>810039497982</v>
+        <v>4</v>
+      </c>
+      <c r="I23" s="3" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A25" s="3" t="s">
-        <v>14</v>
+        <v>21</v>
       </c>
       <c r="B25" s="3">
         <v>1</v>
       </c>
       <c r="C25" s="3" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="D25" s="3" t="s">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="E25" s="3" t="s">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="G25" s="3">
-        <v>9.9</v>
+        <v>34</v>
       </c>
       <c r="H25" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="I25" s="3" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A26" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="B26" s="3">
-        <v>1</v>
-      </c>
-      <c r="C26" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="D26" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="E26" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="G26" s="3">
-        <v>17.5</v>
-      </c>
-      <c r="H26" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="I26" s="3" t="s">
-        <v>28</v>
+        <v>25</v>
+      </c>
+      <c r="I25" s="3">
+        <v>810039497982</v>
       </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A27" s="3" t="s">
-        <v>31</v>
+        <v>14</v>
       </c>
       <c r="B27" s="3">
         <v>1</v>
       </c>
       <c r="C27" s="3" t="s">
-        <v>32</v>
+        <v>17</v>
       </c>
       <c r="D27" s="3" t="s">
         <v>15</v>
       </c>
       <c r="E27" s="3" t="s">
-        <v>33</v>
+        <v>16</v>
       </c>
       <c r="G27" s="3">
-        <v>8.99</v>
+        <v>9.9</v>
       </c>
       <c r="H27" s="3" t="s">
-        <v>34</v>
+        <v>18</v>
       </c>
       <c r="I27" s="3" t="s">
-        <v>35</v>
+        <v>19</v>
       </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A28" s="3" t="s">
-        <v>36</v>
+        <v>26</v>
       </c>
       <c r="B28" s="3">
         <v>1</v>
       </c>
       <c r="C28" s="3" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="D28" s="3" t="s">
         <v>15</v>
       </c>
       <c r="E28" s="3" t="s">
-        <v>38</v>
+        <v>27</v>
       </c>
       <c r="G28" s="3">
-        <v>7.9</v>
+        <v>17.5</v>
       </c>
       <c r="H28" s="3" t="s">
-        <v>39</v>
+        <v>30</v>
       </c>
       <c r="I28" s="3" t="s">
-        <v>40</v>
+        <v>28</v>
       </c>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A29" s="3" t="s">
-        <v>45</v>
+        <v>31</v>
       </c>
       <c r="B29" s="3">
         <v>1</v>
       </c>
       <c r="C29" s="3" t="s">
-        <v>46</v>
+        <v>32</v>
       </c>
       <c r="D29" s="3" t="s">
         <v>15</v>
       </c>
       <c r="E29" s="3" t="s">
-        <v>47</v>
+        <v>33</v>
       </c>
       <c r="G29" s="3">
-        <v>16</v>
+        <v>8.99</v>
       </c>
       <c r="H29" s="3" t="s">
-        <v>48</v>
+        <v>34</v>
       </c>
       <c r="I29" s="3" t="s">
-        <v>49</v>
+        <v>35</v>
       </c>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A30" s="3" t="s">
-        <v>50</v>
+        <v>36</v>
       </c>
       <c r="B30" s="3">
         <v>1</v>
       </c>
       <c r="C30" s="3" t="s">
-        <v>51</v>
+        <v>37</v>
       </c>
       <c r="D30" s="3" t="s">
         <v>15</v>
       </c>
       <c r="E30" s="3" t="s">
-        <v>52</v>
+        <v>38</v>
       </c>
       <c r="G30" s="3">
-        <v>11.8</v>
+        <v>7.9</v>
       </c>
       <c r="H30" s="3" t="s">
-        <v>53</v>
+        <v>39</v>
       </c>
       <c r="I30" s="3" t="s">
-        <v>54</v>
+        <v>40</v>
       </c>
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A31" s="3" t="s">
-        <v>55</v>
+        <v>45</v>
       </c>
       <c r="B31" s="3">
         <v>1</v>
       </c>
       <c r="C31" s="3" t="s">
-        <v>56</v>
+        <v>46</v>
       </c>
       <c r="D31" s="3" t="s">
         <v>15</v>
       </c>
       <c r="E31" s="3" t="s">
-        <v>57</v>
+        <v>47</v>
       </c>
       <c r="G31" s="3">
-        <v>39.5</v>
+        <v>16</v>
       </c>
       <c r="H31" s="3" t="s">
-        <v>58</v>
+        <v>48</v>
       </c>
       <c r="I31" s="3" t="s">
-        <v>59</v>
+        <v>49</v>
       </c>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A32" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="B32" s="3">
+        <v>1</v>
+      </c>
+      <c r="C32" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="D32" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="E32" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="G32" s="3">
+        <v>11.8</v>
+      </c>
+      <c r="H32" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="I32" s="3" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="33" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A33" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="B33" s="3">
+        <v>1</v>
+      </c>
+      <c r="C33" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="D33" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="E33" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="G33" s="3">
+        <v>39.5</v>
+      </c>
+      <c r="H33" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="I33" s="3" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="34" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A34" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="B32" s="3">
-        <v>1</v>
-      </c>
-      <c r="C32" s="3" t="s">
+      <c r="B34" s="3">
+        <v>1</v>
+      </c>
+      <c r="C34" s="3" t="s">
         <v>61</v>
       </c>
-      <c r="D32" s="3" t="s">
+      <c r="D34" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="E32" s="3" t="s">
+      <c r="E34" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="G32" s="3">
+      <c r="G34" s="3">
         <v>9.9499999999999993</v>
       </c>
-      <c r="H32" s="3" t="s">
+      <c r="H34" s="3" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A34" s="3" t="s">
+    <row r="36" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A36" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="B34" s="3">
-        <v>1</v>
-      </c>
-      <c r="C34" s="3" t="s">
+      <c r="B36" s="3">
+        <v>1</v>
+      </c>
+      <c r="C36" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="E34" s="3" t="s">
+      <c r="E36" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="G34" s="3">
+      <c r="G36" s="3">
         <v>70</v>
       </c>
-      <c r="H34" s="4" t="s">
+      <c r="H36" s="4" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="H35" s="4"/>
-    </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="H36" s="4"/>
-    </row>
-    <row r="37" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:9" x14ac:dyDescent="0.35">
       <c r="H37" s="4"/>
     </row>
-    <row r="38" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A38" s="3" t="s">
+    <row r="38" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="H38" s="4"/>
+    </row>
+    <row r="39" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="H39" s="4"/>
+    </row>
+    <row r="40" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A40" s="3" t="s">
         <v>105</v>
       </c>
-      <c r="G38" s="3">
-        <f xml:space="preserve"> SUM(G2:G35)</f>
-        <v>369.71999999999997</v>
+      <c r="G40" s="3">
+        <f xml:space="preserve"> SUM(G2:G37)</f>
+        <v>387.21999999999997</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="H34" r:id="rId1"/>
+    <hyperlink ref="H36" r:id="rId1"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" r:id="rId2"/>

</xml_diff>